<commit_message>
SPR-01 vong sua 1 (A): noi dung - bo ten rieng con sot, con tro Goc nhin, CAMPAIGNS khop workbook, bai mau FB qua cong fb_format, dcterms co dinh
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/sample-course/campaigns.xlsx
+++ b/content/sample-course/campaigns.xlsx
@@ -554,10 +554,10 @@
         <v>1</v>
       </c>
       <c r="L2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N2" t="n">
         <v>1</v>

</xml_diff>